<commit_message>
Update manuscript materials and analyses
</commit_message>
<xml_diff>
--- a/manuscript_material/glossary/Glossary.xlsx
+++ b/manuscript_material/glossary/Glossary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>62 of 100 CompBioBench tasks with one distinct answer across all 12 Galaxy runs</t>
+          <t>One distinct answer in 333 of 400 Galaxy-condition CompBioBench replicate sets; 62 of 100 tasks across all 12 Galaxy runs</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1404,67 +1404,71 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Estimand</t>
+          <t>Replicate agreement</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>New</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>The specific quantity being summarized or compared. Used mainly in Methods.</t>
+          <t>Umbrella term for agreement among the replicate runs of replicate sets: outcome repeatability where a verdict or score exists, answer consistency otherwise.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Condition difference in accuracy</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
+          <t>Section 3 of the Results; Fig. 4</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>reproducibility (for replicate runs)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Analysis process and Galaxy records</t>
+          <t>Outcomes and comparisons</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Analysis trajectory</t>
+          <t>Run-level accuracy; unanimous accuracy</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>New</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>The sequence of analytical actions an agent takes during a run to reach, or attempt to reach, its final answer. It does not imply the answer was scored correct.</t>
+          <t>Run-level accuracy is accuracy over runs. Unanimous accuracy is the share of BixBench-Verified-50 tasks whose three replicate runs were all scored correct (repeatability category 3/3), per model configuration and execution condition. Compare the two only over the same model configurations.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Inspect data → filter → run DESeq2 → inspect output → submit answer</t>
+          <t>GPT-5.5, Galaxy condition: 89.3% run-level, 88.0% unanimous</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>solution path; path</t>
+          <t>strict accuracy; triplicate accuracy</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Analysis process and Galaxy records</t>
+          <t>Outcomes and comparisons</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Execution trace</t>
+          <t>Estimand</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1474,19 +1478,15 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>The recorded evidence documenting an analysis trajectory: agent messages, commands, tool calls, Galaxy jobs and outputs.</t>
+          <t>The specific quantity being summarized or compared. Used mainly in Methods.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Codex trace plus Galaxy history</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>agent trace; transcript</t>
-        </is>
-      </c>
+          <t>Condition difference in accuracy</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Analytical operation</t>
+          <t>Analysis trajectory</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1506,15 +1506,19 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>A scientifically meaningful computational action within an analysis trajectory.</t>
+          <t>The sequence of analytical actions an agent takes during a run to reach, or attempt to reach, its final answer. It does not imply the answer was scored correct.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Alignment, filtering, differential expression, enrichment</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>Inspect data → filter → run DESeq2 → inspect output → submit answer</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>solution path; path</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1524,7 +1528,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tool-set fingerprint</t>
+          <t>Execution trace</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1534,17 +1538,17 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>An unordered set of tool identifiers (Galaxy) or command names (open-ended code) used in a run. It does not encode operation order, parameters or biological decisions.</t>
+          <t>The recorded evidence documenting an analysis trajectory: agent messages, commands, tool calls, Galaxy jobs and outputs.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Set of version-stripped Galaxy tool IDs used in one run</t>
+          <t>Codex trace plus Galaxy history</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>recorded path</t>
+          <t>agent trace; transcript</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1560,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Tool-set similarity</t>
+          <t>Analytical operation</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1566,19 +1570,15 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Overlap between tool-set fingerprints across the replicate runs of a replicate set, measured as mean pairwise Jaccard similarity.</t>
+          <t>A scientifically meaningful computational action within an analysis trajectory.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Mean Galaxy tool-set similarity of 0.616 (IWC) versus 0.134 (CompBioBench)</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>path agreement; Jaccard index</t>
-        </is>
-      </c>
+          <t>Alignment, filtering, differential expression, enrichment</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Declared route</t>
+          <t>Tool-set fingerprint</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1598,15 +1598,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>The analytical method an agent states it used. It is not independently verified and is distinct from the tool-set fingerprint.</t>
+          <t>An unordered set of tool identifiers (Galaxy) or command names (open-ended code) used in a run. It does not encode operation order, parameters or biological decisions.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>DESeq2 versus edgeR for IWC RNA-seq differential expression</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>Set of version-stripped Galaxy tool IDs used in one run</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>recorded path</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1616,27 +1620,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Galaxy interface call</t>
+          <t>Tool-set similarity</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>One call from the agent to Galaxy through the programmatic interface of the Galaxy condition (a Model Context Protocol server), such as a tool search, tool inspection or job submission.</t>
+          <t>Overlap between tool-set fingerprints across the replicate runs of a replicate set, measured as mean pairwise Jaccard similarity.</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>69,812 Galaxy interface calls, of which 7,389 returned a failure status</t>
+          <t>Mean Galaxy tool-set similarity of 0.616 (IWC) versus 0.134 (CompBioBench)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>MCP call</t>
+          <t>path agreement; Jaccard index</t>
         </is>
       </c>
     </row>
@@ -1648,29 +1652,25 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Direct Galaxy API call</t>
+          <t>Declared route</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>A shell command that calls Galaxy's web API or the BioBlend library directly, outside the Galaxy interface.</t>
+          <t>The analytical method an agent states it used. It is not independently verified and is distinct from the tool-set fingerprint.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Copying the provided analysis history in 537 of 600 Codex BixBench Galaxy runs</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>BioBlend or raw REST bypass</t>
-        </is>
-      </c>
+          <t>DESeq2 versus edgeR for IWC RNA-seq differential expression</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Analysis history</t>
+          <t>Galaxy interface call</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1690,17 +1690,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>The Galaxy record (history) of the datasets, jobs, tools and parameters produced during a run.</t>
+          <t>One call from the agent to Galaxy through the programmatic interface of the Galaxy condition (a Model Context Protocol server), such as a tool search, tool inspection or job submission.</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>714 of 750 BixBench Galaxy runs have a detailed analysis-history snapshot</t>
+          <t>69,812 Galaxy interface calls, of which 7,389 returned a failure status</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>history (unqualified)</t>
+          <t>MCP call</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Galaxy analysis job</t>
+          <t>Direct Galaxy API call</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1722,17 +1722,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>A Galaxy job other than a data-fetch (upload) job, counted once per server and job identifier.</t>
+          <t>A shell command that calls Galaxy's web API or the BioBlend library directly, outside the Galaxy interface.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>23,080 Galaxy analysis jobs (5,042 BixBench; 16,686 CompBioBench; 1,352 IWC)</t>
+          <t>Copying the provided analysis history in 537 of 600 Codex BixBench Galaxy runs</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>non-fetch job</t>
+          <t>BioBlend or raw REST bypass</t>
         </is>
       </c>
     </row>
@@ -1744,27 +1744,27 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Installed Galaxy tool</t>
+          <t>Analysis history</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>New</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>A Tool Shed wrapper available on the Galaxy server. Subdivided into domain tools and utility tools.</t>
+          <t>The Galaxy record (history) of the datasets, jobs, tools and parameters produced during a run.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Any wrapper in the server's tool panel</t>
+          <t>714 of 750 BixBench Galaxy runs have a detailed analysis-history snapshot</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>installed wrapper</t>
+          <t>history (unqualified)</t>
         </is>
       </c>
     </row>
@@ -1776,27 +1776,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Domain tool</t>
+          <t>Galaxy analysis job</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>New</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>An installed Galaxy tool implementing a domain-specific analytical method.</t>
+          <t>A Galaxy job other than a data-fetch (upload) job, counted once per server and job identifier.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>fastp, DADA2, PepQuery, Bowtie2</t>
+          <t>23,080 Galaxy analysis jobs (5,042 BixBench; 16,686 CompBioBench; 1,352 IWC)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>domain-analysis tool; non-utility Tool Shed job</t>
+          <t>non-fetch job</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Utility tool</t>
+          <t>Installed Galaxy tool</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1818,17 +1818,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>An installed Galaxy tool for generic data handling.</t>
+          <t>A Tool Shed wrapper available on the Galaxy server. Subdivided into domain tools and utility tools.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Cut, Filter, xlsx2tsv, Datamash</t>
+          <t>Any wrapper in the server's tool panel</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>file or table utility</t>
+          <t>installed wrapper</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>User-defined tool (UDT)</t>
+          <t>Domain tool</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1850,15 +1850,19 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>A custom tool written by the agent and executed through Galaxy's interface.</t>
+          <t>An installed Galaxy tool implementing a domain-specific analytical method.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Custom wrapper for PhyKIT treeness in bix-11-q1</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>fastp, DADA2, PepQuery, Bowtie2</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>domain-analysis tool; non-utility Tool Shed job</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1868,27 +1872,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Probe tool</t>
+          <t>Utility tool</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>A throwaway user-defined tool written only to find out why jobs fail, because Galaxy offers no trial run.</t>
+          <t>An installed Galaxy tool for generic data handling.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1,859 probe-tool calls in 517 of 808 CompBioBench runs that used user-defined tools</t>
+          <t>Cut, Filter, xlsx2tsv, Datamash</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>probe UDT</t>
+          <t>file or table utility</t>
         </is>
       </c>
     </row>
@@ -1900,29 +1904,25 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Parameter substitution</t>
+          <t>User-defined tool (UDT)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>A difference between the parameter values an agent requested in a Galaxy tool-run call and the tool state Galaxy resolved from them (a value replaced, or a requested value dropped). It is either blocked before submission by the benchmark's check or executed.</t>
+          <t>A custom tool written by the agent and executed through Galaxy's interface.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>4,352 tool-run calls, 916 executed (for example, Datamash max → count)</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>parameter mismatch; requested-versus-resolved difference</t>
-        </is>
-      </c>
+          <t>Custom wrapper for PhyKIT treeness in bix-11-q1</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1932,27 +1932,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Operational error</t>
+          <t>Probe tool</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>New</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>A failed computational operation during a run. It does not by itself imply that the final answer was scored incorrect. Always reported through one of its two instrument-specific subtypes.</t>
+          <t>A throwaway user-defined tool written only to find out why jobs fail, because Galaxy offers no trial run.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Galaxy job error; nonzero shell exit</t>
+          <t>1,859 probe-tool calls in 517 of 808 CompBioBench runs that used user-defined tools</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>failure (for operations)</t>
+          <t>probe UDT</t>
         </is>
       </c>
     </row>
@@ -1964,27 +1964,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Galaxy job error</t>
+          <t>Parameter substitution</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Sharpened</t>
+          <t>New</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>A Galaxy analysis job that ends in error state. Not comparable with nonzero shell exits.</t>
+          <t>A difference between the parameter values an agent requested in a Galaxy tool-run call and the tool state Galaxy resolved from them (a value replaced, or a requested value dropped). It is either blocked before submission by the benchmark's check or executed.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>552 of 5,042 BixBench Galaxy analysis jobs</t>
+          <t>4,352 tool-run calls, 916 executed (for example, Datamash max → count)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>error job; failed job</t>
+          <t>parameter mismatch; requested-versus-resolved difference</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Nonzero shell exit</t>
+          <t>Operational error</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2006,17 +2006,17 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A shell command that returns a nonzero exit code. It can reflect probes or searches rather than analytical failure.</t>
+          <t>A failed computational operation during a run. It does not by itself imply that the final answer was scored incorrect. Always reported through one of its two instrument-specific subtypes.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Failed package check or empty search result</t>
+          <t>Galaxy job error; nonzero shell exit</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>failed shell command</t>
+          <t>failure (for operations)</t>
         </is>
       </c>
     </row>
@@ -2028,27 +2028,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Candidate recovery</t>
+          <t>Galaxy job error</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>Sharpened</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>An operational error followed by a later successful related action, not yet manually adjudicated. This is the default term.</t>
+          <t>A Galaxy analysis job that ends in error state. Not comparable with nonzero shell exits.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>93 candidate recoveries in BixBench</t>
+          <t>552 of 5,042 BixBench Galaxy analysis jobs</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>recovery (unqualified)</t>
+          <t>error job; failed job</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Verified recovery</t>
+          <t>Nonzero shell exit</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2070,15 +2070,19 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>A candidate recovery that manual review confirms: the agent overcame the failure while keeping the same analytical objective.</t>
+          <t>A shell command that returns a nonzero exit code. It can reflect probes or searches rather than analytical failure.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>String columns cast to numeric before a repeated calculation (bedtools-chromhmm-q1)</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
+          <t>Failed package check or empty search result</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>failed shell command</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2088,7 +2092,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Input-token usage</t>
+          <t>Candidate recovery</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2098,17 +2102,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Input tokens consumed by a run or run population, according to archived usage records (cached input included; output and reasoning tokens not added).</t>
+          <t>An operational error followed by a later successful related action, not yet manually adjudicated. This is the default term.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Median of 1.19 million input tokens per GPT-5.5 Galaxy run on BixBench</t>
+          <t>93 candidate recoveries in BixBench</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>input tokens; token burden</t>
+          <t>recovery (unqualified)</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2124,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Input-token ratio</t>
+          <t>Verified recovery</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2130,79 +2134,79 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Median Galaxy input-token usage divided by median open-ended code input-token usage, for the same task and model configuration.</t>
+          <t>A candidate recovery that manual review confirms: the agent overcame the failure while keeping the same analytical objective.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Median ratio of 4.74 on BixBench</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>token overhead; token multiplier</t>
-        </is>
-      </c>
+          <t>String columns cast to numeric before a repeated calculation (bedtools-chromhmm-q1)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Adjudication</t>
+          <t>Analysis process and Galaxy records</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Primary cause; secondary cause</t>
+          <t>Input-token usage</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>The main reason, and at most one contributing reason, for a scored-incorrect run (or an IWC run with output agreement below 0.5), assigned by trace-level adjudication from seven categories: task under-specified or reference ambiguous; statistical or reasoning error; evaluator rejected a correct answer; missing domain knowledge; platform or tool defect; no answer submitted; output format violated.</t>
+          <t>Input tokens consumed by a run or run population, according to archived usage records (cached input included; output and reasoning tokens not added).</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Galaxy platform or tool defect: primary in 4 and secondary in 18 of 111 scored-incorrect Galaxy runs</t>
+          <t>Median of 1.19 million input tokens per GPT-5.5 Galaxy run on BixBench</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>root cause</t>
+          <t>input tokens; token burden</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Adjudication</t>
+          <t>Analysis process and Galaxy records</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Adjudication confidence</t>
+          <t>Input-token ratio</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>How firmly the decisive step of a scored-incorrect run was established: high, moderate, mixed or unresolved (Supplementary Note 6).</t>
+          <t>Median Galaxy input-token usage divided by median open-ended code input-token usage, for the same task and model configuration.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>159 high, 55 moderate, 20 mixed and 12 unresolved of 246 BixBench adjudications</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
+          <t>Median ratio of 4.74 on BixBench</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>token overhead; token multiplier</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2212,7 +2216,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Divergence mechanism</t>
+          <t>Task case</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2222,15 +2226,19 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>What separated a scored-incorrect replicate run from its scored-correct sibling(s) in a split replicate set. Distinct from its primary cause.</t>
+          <t>A task with at least one wrong, scored-incorrect or low-scoring run (plus one IWC workflow whose near-perfect output agreement concealed a changed result), audited across all of its runs. The unit of the task-level audit; each task is counted once.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Hand-written method or software-version difference: 30 of 45 open-ended code runs versus 5 of 36 Galaxy runs</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>93 task cases: 33 BixBench-Verified-50, 53 CompBioBench, 7 IWC</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>failed task; error case</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2240,25 +2248,305 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
+          <t>Primary cause category (task case)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>The main interpretive issue of a task case, one of eight: C1 equivalent answer expressed differently; C2 scoring or evaluator artifact; C3 reference depends on an unstated choice; C4 Galaxy platform, wrapper or server behaviour; C5 agent analysis error; C6 execution provenance or answer exposure; C7 aggregate score conceals a changed scientific conclusion; C8 completion failure. C1–C3 place the cause with the benchmark.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>C3, reference depends on an unstated choice: 20 of 93 task cases</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>root cause (for tasks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Integrity flag</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>A problem with how an answer was obtained, recorded in addition to the primary cause: benchmark-answer retrieval, local computation in the Galaxy condition or cross-run output reuse. A flag does not imply that the answer is wrong.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Benchmark-answer retrieval in 26 of 93 task cases</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>contamination (unqualified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Benchmark-answer retrieval</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>An agent retrieved, or tried to retrieve, a benchmark answer or a source that fixes it (the benchmark key, another agent's answer, a source paper or dataset) from the web during a run.</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>10 task cases in which a benchmark answer, the key or another agent's answer was obtained</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>answer leakage; cheating</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Local computation (Galaxy condition)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>A Galaxy-condition run whose decisive computation ran in the local shell, with the result only staged into Galaxy, typically after user-defined-tool execution became unavailable on the server. The run keeps its condition label but is not counted as execution within Galaxy.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>15 scored-correct and 3 scored-incorrect CompBioBench Galaxy-condition runs</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>local fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Cross-run output reuse</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>A run that obtained its answer from the analysis history or job outputs of another run through the shared Galaxy account.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>GPT-5.6 Luna, encode-atac-pipeline-q1, Galaxy condition, replicate run 1</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>answer copying</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Interface-binding failure</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>An executed parameter substitution that changes the analysis: Galaxy binds the requested tool state to a different option (for example the default of a nested conditional) and the job succeeds, so no error is returned.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>bix-35-q1: PhyKIT ran "total tree length" instead of "evolutionary rate"</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>silent default (unqualified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Primary cause; secondary cause</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Run level (failure ledger): the main reason, and at most one contributing reason, for a scored-incorrect run (or an IWC run with output agreement below 0.5), assigned by trace-level adjudication from seven categories: task under-specified or reference ambiguous; statistical or reasoning error; evaluator rejected a correct answer; missing domain knowledge; platform or tool defect; no answer submitted; output format violated.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Galaxy platform or tool defect: primary in 4 and secondary in 18 of 111 scored-incorrect Galaxy runs</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>root cause</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Adjudication confidence</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>How firmly the decisive step of a scored-incorrect run was established: high, moderate, mixed or unresolved (Supplementary Note 6).</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>159 high, 55 moderate, 20 mixed and 12 unresolved of 246 BixBench adjudications</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Divergence mechanism</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>What separated a scored-incorrect replicate run from its scored-correct sibling(s) in a split replicate set. Distinct from its primary cause.</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Hand-written method or software-version difference: 30 of 45 open-ended code runs versus 5 of 36 Galaxy runs</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Adjudication</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>Verifier mode</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>The rule the BixBench evaluator uses to compare a numeric answer with the reference: tolerance (within a stated margin) or rounded-numeric (after rounding).</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>bix-43-q2: 5.831005… scored correct under the tolerance verifier and incorrect under the rounded-numeric verifier</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>